<commit_message>
Add 4 archive categories + refresh import template
New categories: Photography & Posters, Film & Movies, Family Archives,
Trade & Sports Cards (migration 005). Bulk-import template's category dropdown
and Instructions updated to match (now 16 categories).

Run 005_more_categories.sql in the member-app Supabase project to activate.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/preston-archive-import-template.xlsx
+++ b/templates/preston-archive-import-template.xlsx
@@ -907,7 +907,7 @@
     <row r="40">
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Fine Art · Jewelry · Coins &amp; Numismatics · Horology · Manuscripts · Sports Memorabilia · Stamps &amp; Philately · Militaria · Ceramics &amp; Glass · Rare Books · Furniture &amp; Decor · Ephemera &amp; Documents</t>
+          <t>Fine Art · Jewelry · Coins &amp; Numismatics · Horology · Manuscripts · Sports Memorabilia · Stamps &amp; Philately · Militaria · Ceramics &amp; Glass · Rare Books · Furniture &amp; Decor · Ephemera &amp; Documents · Photography &amp; Posters · Film &amp; Movies · Family Archives · Trade &amp; Sports Cards</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
   </sheetData>
   <dataValidations count="6">
     <dataValidation sqref="C3:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>"Fine Art,Jewelry,Coins &amp; Numismatics,Horology,Manuscripts,Sports Memorabilia,Stamps &amp; Philately,Militaria,Ceramics &amp; Glass,Rare Books,Furniture &amp; Decor,Ephemera &amp; Documents"</formula1>
+      <formula1>"Fine Art,Jewelry,Coins &amp; Numismatics,Horology,Manuscripts,Sports Memorabilia,Stamps &amp; Philately,Militaria,Ceramics &amp; Glass,Rare Books,Furniture &amp; Decor,Ephemera &amp; Documents,Photography &amp; Posters,Film &amp; Movies,Family Archives,Trade &amp; Sports Cards"</formula1>
     </dataValidation>
     <dataValidation sqref="U3:U1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>"TRUE,FALSE"</formula1>

</xml_diff>